<commit_message>
Thêm thành viên Nguyễn Đặng Thành Vinh (2A202602021)
- README: thêm dòng trong bảng thành viên, phần phụ trách (kiến trúc
  tin cậy + thu thập bằng chứng) và góp ý cho Nhóm 05 ở trục Hành động
- Dashboard v2: chuyển 2 chỉ số tin cậy/bàn giao sang owner Vinh,
  cổng 31-60 ngày do Vinh phụ trách, cổng 61-90 chuyển cho Hùng
- Memo: cập nhật bảng owner của lộ trình 30-60-90

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -585,7 +585,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Nhóm Đức·Hùng (Đỗ Quý Đức 2A202601628 · Nguyễn Thanh Hùng 2A202601808)  |  Quyết định: SỬA — pilot 90 ngày trên 1 nhóm, chưa rollout rộng</t>
+          <t>Nhóm Đức·Hùng·Vinh (Đỗ Quý Đức 2A202601628 · Nguyễn Thanh Hùng 2A202601808 · Nguyễn Đặng Thành Vinh 2A202602021)  |  Quyết định: SỬA — pilot 90 ngày trên 1 nhóm, chưa rollout rộng</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thanh Hùng (phụ trách QA)</t>
+          <t>Nguyễn Đặng Thành Vinh (phụ trách kiến trúc tin cậy)</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thanh Hùng (phụ trách AI/QA)</t>
+          <t>Nguyễn Đặng Thành Vinh (phụ trách kiến trúc tin cậy)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1029,7 +1029,7 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Kiểm: 3 chỉ số cấp Product · 3 chỉ số cấp Workflow · 1 chỉ số Business — phủ đủ 5 tầng đo lường.</t>
+          <t>Kiểm: 3 chỉ số cấp Product · 3 chỉ số cấp Workflow · 1 chỉ số Business — phủ đủ 5 tầng đo lường. Owner: Đỗ Quý Đức 3 chỉ số (quy trình &amp; nghiệp vụ) · Nguyễn Thanh Hùng 2 (hành vi &amp; QA) · Nguyễn Đặng Thành Vinh 2 (tin cậy &amp; bàn giao).</t>
         </is>
       </c>
     </row>
@@ -1911,8 +1911,8 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Thanh Hùng
-(QA + đo lường)</t>
+          <t>Nguyễn Đặng Thành Vinh
+(kiến trúc tin cậy)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1950,8 +1950,8 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Đỗ Quý Đức
-(báo cáo trưởng nhóm vận hành)</t>
+          <t>Nguyễn Thanh Hùng
+(đo lường; báo cáo trưởng nhóm vận hành)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">

</xml_diff>